<commit_message>
initial dataset and image processing pipeline
</commit_message>
<xml_diff>
--- a/data/quality_assessment/annotations/quality_dataset.xlsx
+++ b/data/quality_assessment/annotations/quality_dataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FloraSense_Quality_Assessment\dataset\annotations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ResearchProject\J26-DS-332-FloraSense\data\quality_assessment\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A55BBE-3042-4623-AA98-5D813E56DBEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DC43D9-FDD1-4FC1-B37A-5677CD8DFB1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
   </bookViews>
   <sheets>
     <sheet name="Plant_Types" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="141">
   <si>
     <t>Plant_ID</t>
   </si>
@@ -464,6 +464,9 @@
   </si>
   <si>
     <t>data/quality_assessment/original/individual/P01/P01_S019_root.jpg</t>
+  </si>
+  <si>
+    <t>Min_Total_Leaf_Count</t>
   </si>
 </sst>
 </file>
@@ -935,16 +938,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83CB1C05-2934-4DAD-8813-2F1EFF28426D}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="4" width="16.5546875" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" customWidth="1"/>
-    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="2" max="5" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
+    <col min="7" max="7" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -958,16 +961,19 @@
         <v>25</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -980,17 +986,20 @@
       <c r="D2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="3">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2">
         <v>20</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>25</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -1003,13 +1012,16 @@
       <c r="D3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="3">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2">
         <v>30</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>35</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
P01 image-based leaf height measurement prototype
</commit_message>
<xml_diff>
--- a/data/quality_assessment/annotations/quality_dataset.xlsx
+++ b/data/quality_assessment/annotations/quality_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ResearchProject\J26-DS-332-FloraSense\data\quality_assessment\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE10E0D-64FD-4BBE-9328-7098F0ACD987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA6D7937-00C1-4207-BD7D-FF08643E6BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
+    <workbookView xWindow="10464" yWindow="1752" windowWidth="12576" windowHeight="10488" firstSheet="2" activeTab="3" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
   </bookViews>
   <sheets>
     <sheet name="Plant_Types" sheetId="1" r:id="rId1"/>
@@ -1019,10 +1019,10 @@
         <v>8</v>
       </c>
       <c r="F3" s="2">
+        <v>25</v>
+      </c>
+      <c r="G3" s="2">
         <v>30</v>
-      </c>
-      <c r="G3" s="2">
-        <v>35</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
add baseline error analysis and annotation guidelines
</commit_message>
<xml_diff>
--- a/data/quality_assessment/annotations/quality_dataset.xlsx
+++ b/data/quality_assessment/annotations/quality_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ResearchProject\J26-DS-332-FloraSense\data\quality_assessment\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE0A253-F003-4EEE-ADE7-CDE125F6BE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EE24C8-269D-4602-ABC2-E84BE7C0BB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
+    <workbookView xWindow="10464" yWindow="1752" windowWidth="12576" windowHeight="10488" firstSheet="4" activeTab="4" xr2:uid="{3BCCBFA2-B037-441A-851A-B4F452200103}"/>
   </bookViews>
   <sheets>
     <sheet name="Plant_Types" sheetId="1" r:id="rId1"/>
@@ -10724,7 +10724,7 @@
         <v>338</v>
       </c>
       <c r="E83" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F83" t="s">
         <v>17</v>
@@ -10733,7 +10733,7 @@
         <v>86</v>
       </c>
       <c r="H83" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
@@ -11114,7 +11114,7 @@
         <v>340</v>
       </c>
       <c r="E98" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F98" t="s">
         <v>17</v>
@@ -11123,7 +11123,7 @@
         <v>86</v>
       </c>
       <c r="H98" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
@@ -11400,7 +11400,7 @@
         <v>340</v>
       </c>
       <c r="E109" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F109" t="s">
         <v>17</v>

</xml_diff>